<commit_message>
Update Valid Anagram progress in Excel and README
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -779,22 +779,54 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="11" t="n"/>
-      <c r="N5" s="11" t="n"/>
-      <c r="O5" s="11" t="n"/>
-      <c r="P5" s="11" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Create 2 unordered maps to count frequencies and compare</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>Missed single-map optimization; vector index subtraction trick was unknown</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>Single map (increment/decrement) and fixed-size vector of size 26 using char - 'a'</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P5" s="11" t="n">
+        <v>3.5</v>
+      </c>
       <c r="Q5" s="11" t="n"/>
-      <c r="R5" s="11" t="n"/>
+      <c r="R5" s="11" t="inlineStr">
+        <is>
+          <t>Remember how to use a fixed-size array/vector for counting character frequencies</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">

</xml_diff>

<commit_message>
Update Group Anagrams progress in Excel and README
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -859,22 +859,54 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="n"/>
-      <c r="K6" s="11" t="n"/>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="11" t="n"/>
-      <c r="N6" s="11" t="n"/>
-      <c r="O6" s="11" t="n"/>
-      <c r="P6" s="11" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>Brute force nested loops comparing all word pairs using anagram check</t>
+        </is>
+      </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>Index out-of-bounds in nested loops, naming conflict with std::map, missed map grouping structure</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>Sort each word to make a canonical key, and group using unordered_map&lt;string, vector&lt;string&gt;&gt;</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>O(N * L log L)</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>O(N * L)</t>
+        </is>
+      </c>
+      <c r="P6" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="Q6" s="11" t="n"/>
-      <c r="R6" s="11" t="n"/>
+      <c r="R6" s="11" t="inlineStr">
+        <is>
+          <t>Use unordered_map&lt;K, vector&lt;T&gt;&gt; to group items of type T by property K. Avoid naming variables 'map' due to std::map conflicts.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">

</xml_diff>

<commit_message>
Update Two Sum II progress in Excel and README
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -987,22 +987,54 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
-      <c r="O8" s="11" t="n"/>
-      <c r="P8" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>Two pointers from start and end, check sum, increment start or decrement end</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>Index vs value mixup initially, minor warning on return type</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>Two-pointer technique on sorted array using start and end indices</t>
+        </is>
+      </c>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="Q8" s="11" t="n"/>
-      <c r="R8" s="11" t="n"/>
+      <c r="R8" s="11" t="inlineStr">
+        <is>
+          <t>Remember difference between -&gt; and . operators (-&gt; for pointers/iterators, . for direct objects)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">

</xml_diff>

<commit_message>
Update Best Time to Buy and Sell Stock progress in Excel and README
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1067,22 +1067,54 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="11" t="n"/>
-      <c r="M9" s="11" t="n"/>
-      <c r="N9" s="11" t="n"/>
-      <c r="O9" s="11" t="n"/>
-      <c r="P9" s="11" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Try to maintain only 2 pointers for buy and sell day, but couldn't handle shifting minimums without losing historical max profit</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>Did not track the max historical profit separately from the current minimum buy price; got stuck on variable initialization</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>Greedy/Running Minimum. Track the minimum price seen so far, and update the max profit whenever today's price minus the min price exceeds the previous max profit</t>
+        </is>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O9" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P9" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="Q9" s="11" t="n"/>
-      <c r="R9" s="11" t="n"/>
+      <c r="R9" s="11" t="inlineStr">
+        <is>
+          <t>Use running minimum to track the best buy day and record max profit. Don't lose historical max profit when updating the current minimum.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">

</xml_diff>

<commit_message>
Solve Problem 9 (Running Sum) and Problem 10 (Subarray Sum Equals K)
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1147,22 +1147,54 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="11" t="n"/>
-      <c r="M10" s="11" t="n"/>
-      <c r="N10" s="11" t="n"/>
-      <c r="O10" s="11" t="n"/>
-      <c r="P10" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>Keep a running sum variable and update each element in-place</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>Initial += arithmetic typo adding element twice</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>Prefix Sum in-place in O(N) time and O(1) space</t>
+        </is>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P10" s="11" t="n">
+        <v>5</v>
+      </c>
       <c r="Q10" s="11" t="n"/>
-      <c r="R10" s="11" t="n"/>
+      <c r="R10" s="11" t="inlineStr">
+        <is>
+          <t>Modify array in-place to get running sum with O(1) extra space.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
@@ -1195,22 +1227,54 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
-      <c r="L11" s="11" t="n"/>
-      <c r="M11" s="11" t="n"/>
-      <c r="N11" s="11" t="n"/>
-      <c r="O11" s="11" t="n"/>
-      <c r="P11" s="11" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Two pointers / sliding window</t>
+        </is>
+      </c>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>Negative numbers break sliding window; set missed multiple frequency prefix sums</t>
+        </is>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>Prefix Sum + Hash Map. Subarray sum = current_sum - previous_sum = k</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O11" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="P11" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="Q11" s="11" t="n"/>
-      <c r="R11" s="11" t="n"/>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>Use unordered_map&lt;int, int&gt; to store frequency of prefix sums. Check complement sum-k BEFORE inserting current sum.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 11 Minimum Size Subarray Sum using Variable Sliding Window
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1310,13 +1310,29 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
-      <c r="L12" s="11" t="n"/>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Solved</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>Initial attempt used Prefix Sum + Map (solves exact sum = k). For positive integers with sum &gt;= target, use Two-Pointer Sliding Window expanding 'right' and shrinking 'left' in O(N) time and O(1) space.</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
+          <t>Missed strictly positive property and tried single while loop with complex bounds. Learned standard for (right) + while (left) sliding window structure.</t>
+        </is>
+      </c>
       <c r="M12" s="11" t="n"/>
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>

</xml_diff>

<commit_message>
Solve No. 12 Longest Substring Without Repeating Characters with generic template
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1374,13 +1374,29 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="H13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>Solved</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Don't waste memory or calculations manually maintaining length in a sliding window with length++ / length--. Since both back and front pointers are inclusive, the window length is always simply (front - back + 1). Use max(longest, front - back + 1). Implemented generic C++ template for any container (strings and vectors).</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>Tried manual length tracking and if/else insert bug where duplicate was erased but new character was never inserted. Fixed with clean while(set.count) + unconditional insert pattern.</t>
+        </is>
+      </c>
       <c r="M13" s="11" t="n"/>
       <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>

</xml_diff>

<commit_message>
Solve No. 13: Permutation in String (Sliding Window + Frequency Matching) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1307,38 +1307,58 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
           <t>Solved</t>
         </is>
       </c>
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>Initial attempt used Prefix Sum + Map (solves exact sum = k). For positive integers with sum &gt;= target, use Two-Pointer Sliding Window.</t>
+        </is>
+      </c>
+      <c r="L12" s="11" t="inlineStr">
+        <is>
+          <t>Missed strictly positive property and tried complex single while loop.</t>
+        </is>
+      </c>
+      <c r="M12" s="11" t="inlineStr">
+        <is>
+          <t>Standard Variable Sliding Window: expand right, shrink left while windowSum &gt;= target.</t>
+        </is>
+      </c>
+      <c r="N12" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O12" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P12" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q12" s="11" t="inlineStr">
+        <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="J12" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>Initial attempt used Prefix Sum + Map (solves exact sum = k). For positive integers with sum &gt;= target, use Two-Pointer Sliding Window expanding 'right' and shrinking 'left' in O(N) time and O(1) space.</t>
-        </is>
-      </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>Missed strictly positive property and tried single while loop with complex bounds. Learned standard for (right) + while (left) sliding window structure.</t>
-        </is>
-      </c>
-      <c r="M12" s="11" t="n"/>
-      <c r="N12" s="11" t="n"/>
-      <c r="O12" s="11" t="n"/>
-      <c r="P12" s="11" t="n"/>
-      <c r="Q12" s="11" t="n"/>
-      <c r="R12" s="11" t="n"/>
+      <c r="R12" s="11" t="inlineStr">
+        <is>
+          <t>For strictly positive numbers, sliding window expanding right and shrinking left gives O(N) time and O(1) space.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n">
@@ -1371,38 +1391,58 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
           <t>Solved</t>
         </is>
       </c>
+      <c r="H13" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Track character set and sliding window length.</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>Tried manual length tracking with length++/length-- and if/else insert bug.</t>
+        </is>
+      </c>
+      <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>Variable sliding window with unordered_set: while(set.count) erase(left++), then insert(right) and update max(longest, right - left + 1). Generic C++ template.</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>O(min(N, Sigma))</t>
+        </is>
+      </c>
+      <c r="P13" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="11" t="inlineStr">
+        <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="J13" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>Don't waste memory or calculations manually maintaining length in a sliding window with length++ / length--. Since both back and front pointers are inclusive, the window length is always simply (front - back + 1). Use max(longest, front - back + 1). Implemented generic C++ template for any container (strings and vectors).</t>
-        </is>
-      </c>
-      <c r="L13" s="11" t="inlineStr">
-        <is>
-          <t>Tried manual length tracking and if/else insert bug where duplicate was erased but new character was never inserted. Fixed with clean while(set.count) + unconditional insert pattern.</t>
-        </is>
-      </c>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n"/>
-      <c r="O13" s="11" t="n"/>
-      <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="11" t="n"/>
-      <c r="R13" s="11" t="n"/>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>Don't waste memory/calculations maintaining length manually in sliding window. Both pointers inclusive gives (front - back + 1).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n">
@@ -1435,22 +1475,58 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n"/>
-      <c r="M14" s="11" t="n"/>
-      <c r="N14" s="11" t="n"/>
-      <c r="O14" s="11" t="n"/>
-      <c r="P14" s="11" t="n"/>
-      <c r="Q14" s="11" t="n"/>
-      <c r="R14" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>Vector of size 26 for char frequency match; initially feared vector comparison inside loop would be O(N^2).</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Missing -'a' ASCII offset causing vector out-of-bounds assert, and missing final window check after loop exit.</t>
+        </is>
+      </c>
+      <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>Fixed-size sliding window (size |s1|). Compare 26-char frequency vectors in O(1) time per slide: decrement outgoing s2[back]-'a', increment incoming s2[back+|s1|]-'a'.</t>
+        </is>
+      </c>
+      <c r="N14" s="11" t="inlineStr">
+        <is>
+          <t>O(|s1| + |s2|)</t>
+        </is>
+      </c>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>O(1) (26 chars)</t>
+        </is>
+      </c>
+      <c r="P14" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="inlineStr">
+        <is>
+          <t>Comparing fixed-size frequency vectors (size 26) is always O(1) constant time, making sliding window string permutation check O(N) linear time and O(1) space. Always guard s1.size() &gt; s2.size().</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 14: Valid Parentheses (Stack LIFO matching) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1559,22 +1559,58 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11" t="n"/>
-      <c r="L15" s="11" t="n"/>
-      <c r="M15" s="11" t="n"/>
-      <c r="N15" s="11" t="n"/>
-      <c r="O15" s="11" t="n"/>
-      <c r="P15" s="11" t="n"/>
-      <c r="Q15" s="11" t="n"/>
-      <c r="R15" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>Use stack to store opening brackets and map closing to opening brackets.</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>Calling stack.top() on empty stack when string starts with closing bracket like ']'.</t>
+        </is>
+      </c>
+      <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>Stack + HashMap: push opening brackets, on closing bracket guard stack.empty() before checking stack.top() == brackets[ch], then pop. Finally return stack.empty().</t>
+        </is>
+      </c>
+      <c r="N15" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="P15" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="inlineStr">
+        <is>
+          <t>Nothing much, this was an easy one. LIFO Stack + HashMap matching. Always guard against calling stack.top() on an empty stack when input starts with a closing bracket.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 15: Min Stack (O(1) auxiliary minimum stack design) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1643,22 +1643,58 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="11" t="n"/>
-      <c r="L16" s="11" t="n"/>
-      <c r="M16" s="11" t="n"/>
-      <c r="N16" s="11" t="n"/>
-      <c r="O16" s="11" t="n"/>
-      <c r="P16" s="11" t="n"/>
-      <c r="Q16" s="11" t="n"/>
-      <c r="R16" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>Mapped s.size() to current smallest element using unordered_map.</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>unordered_map has hashing/allocation overhead and double push/pop bugs in draft.</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>Two-stack pattern: maintain parallel minimum stack (or stack of pairs) to track min at each height in O(1) time and O(N) space.</t>
+        </is>
+      </c>
+      <c r="N16" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="O16" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="P16" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr">
+        <is>
+          <t>you can store the minimum entry with map&lt;vector &lt; stack</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 16: Binary Search (Safe mid calculation & space halving) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1727,22 +1727,58 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11" t="n"/>
-      <c r="L17" s="11" t="n"/>
-      <c r="M17" s="11" t="n"/>
-      <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="11" t="n"/>
-      <c r="R17" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>Standard two-pointer search halving low and high.</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="inlineStr">
+        <is>
+          <t>Initially placed mid calculation outside while loop causing infinite loop.</t>
+        </is>
+      </c>
+      <c r="M17" s="11" t="inlineStr">
+        <is>
+          <t>Recalculate mid inside while(low &lt;= high) using safe formula low + (high - low) / 2 to prevent 32-bit integer overflow.</t>
+        </is>
+      </c>
+      <c r="N17" s="11" t="inlineStr">
+        <is>
+          <t>O(log N)</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P17" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="inlineStr">
+        <is>
+          <t>Adding half the distance (high - low) / 2 to low prevents 32-bit integer overflow compared to (low + high) / 2. Always recalculate mid inside the while loop.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 17: Find First and Last Position of Element in Sorted Array (Boundary Binary Search) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1811,22 +1811,58 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H18" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="11" t="n"/>
-      <c r="L18" s="11" t="n"/>
-      <c r="M18" s="11" t="n"/>
-      <c r="N18" s="11" t="n"/>
-      <c r="O18" s="11" t="n"/>
-      <c r="P18" s="11" t="n"/>
-      <c r="Q18" s="11" t="n"/>
-      <c r="R18" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>Find element then search left and right boundaries using separate helper functions.</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>Custom while condition v[leftmost-1] != element caused v[-1] out of bounds crash; also while(left &lt; right) skipped edge index.</t>
+        </is>
+      </c>
+      <c r="M18" s="11" t="inlineStr">
+        <is>
+          <t>Leftmost and Rightmost boundary binary search. Move right = mid - 1 for leftmost search and left = mid + 1 for rightmost search when v[mid] == element. Use while(left &lt;= right).</t>
+        </is>
+      </c>
+      <c r="N18" s="11" t="inlineStr">
+        <is>
+          <t>O(log N)</t>
+        </is>
+      </c>
+      <c r="O18" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P18" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="inlineStr">
+        <is>
+          <t>Leftmost and Rightmost boundary binary search. Move right = mid - 1 for leftmost search and left = mid + 1 for rightmost search when v[mid] == element. Use while(left &lt;= right) to prevent skipping edge indices.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 18: Search in Rotated Sorted Array (Pivot Binary Search) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1895,22 +1895,58 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
-      <c r="L19" s="11" t="n"/>
-      <c r="M19" s="11" t="n"/>
-      <c r="N19" s="11" t="n"/>
-      <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="11" t="n"/>
-      <c r="R19" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Compare mid to right to find pivot, or compare left to mid to identify sorted subarray.</t>
+        </is>
+      </c>
+      <c r="L19" s="11" t="inlineStr">
+        <is>
+          <t>Uninitialized mid and missing left/right pointer updates in while loop caused infinite loop.</t>
+        </is>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>Pass 1: Compare v[left] &lt;= v[mid] to find sorted half and check if target is in that range. Pass 2: Binary search pivot (v[mid] &gt; v[right]), select target half, then binary search.</t>
+        </is>
+      </c>
+      <c r="N19" s="11" t="inlineStr">
+        <is>
+          <t>O(log N)</t>
+        </is>
+      </c>
+      <c r="O19" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P19" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q19" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="inlineStr">
+        <is>
+          <t>You don't always need something out of the box, just check out the edge or different cases. Sometimes they give you a hint: like in this problem, if I compared mid to right I could have known which side has pivot; if I compared left to mid I could have known if the subarray is sorted, and if a subarray is sorted I could check if target exists in that sorted subarray.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 19: Koko Eating Bananas (Binary Search on Answer Space) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -1979,22 +1979,58 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11" t="n"/>
-      <c r="L20" s="11" t="n"/>
-      <c r="M20" s="11" t="n"/>
-      <c r="N20" s="11" t="n"/>
-      <c r="O20" s="11" t="n"/>
-      <c r="P20" s="11" t="n"/>
-      <c r="Q20" s="11" t="n"/>
-      <c r="R20" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>Calculated total_bananas / hrs and maxPile as bounds.</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="inlineStr">
+        <is>
+          <t>Initially missed that range of answer speeds [1 ... maxPile] can be binary searched, and returned mid instead of low.</t>
+        </is>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>Binary Search on Answer Space: binary search speed k in range [1 ... max(piles)] using integer ceil formula (p + k - 1) / k. If totalHrs &lt;= h, set high = mid; else low = mid + 1.</t>
+        </is>
+      </c>
+      <c r="N20" s="11" t="inlineStr">
+        <is>
+          <t>O(N log(max(piles)))</t>
+        </is>
+      </c>
+      <c r="O20" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P20" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>try thinking of binary search if you see upper and lower bound for the range of answer</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 20: Reverse Linked List (3-Pointer Iterative Reversal) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -2067,18 +2067,54 @@
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="11" t="n"/>
-      <c r="L21" s="11" t="n"/>
-      <c r="M21" s="11" t="n"/>
-      <c r="N21" s="11" t="n"/>
-      <c r="O21" s="11" t="n"/>
-      <c r="P21" s="11" t="n"/>
-      <c r="Q21" s="11" t="n"/>
-      <c r="R21" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>Use 3 pointers back, current, and front.</t>
+        </is>
+      </c>
+      <c r="L21" s="11" t="inlineStr">
+        <is>
+          <t>Initially used while(front==nullptr) and accessed front-&gt;val on null causing segmentation fault.</t>
+        </is>
+      </c>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>3-Pointer Iterative Reversal: save next (front = current-&gt;next), flip arrow (current-&gt;next = back), shift pointers (back = current, current = front). Repeat while current != nullptr. Return back as new head.</t>
+        </is>
+      </c>
+      <c r="N21" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O21" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P21" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>save the tommorrow , change direction today and then change move the refrences</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 21: Merge Two Sorted Lists (Dummy Node & Splicing Pattern) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -2147,22 +2147,58 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="11" t="n"/>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="11" t="n"/>
-      <c r="L22" s="11" t="n"/>
-      <c r="M22" s="11" t="n"/>
-      <c r="N22" s="11" t="n"/>
-      <c r="O22" s="11" t="n"/>
-      <c r="P22" s="11" t="n"/>
-      <c r="Q22" s="11" t="n"/>
-      <c r="R22" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>Loop through lists using raw tail and pointers</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>Iterating till end when one list reached null, handling head edge cases and nullptr dereference</t>
+        </is>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>Dummy Node + Splicing: compare list1 and list2 heads, attach smaller node to current-&gt;next, advance current and chosen list. When one list becomes null, attach remaining list directly in O(1).</t>
+        </is>
+      </c>
+      <c r="N22" s="11" t="inlineStr">
+        <is>
+          <t>O(N + M)</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P22" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q22" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="inlineStr">
+        <is>
+          <t>in list you dont need to itterate till end , if one reach null ptr just attach the other one at the current end</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 22: Linked List Cycle (Fast & Slow Pointers and Cycle Entry Detection) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -2231,22 +2231,58 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="n"/>
-      <c r="K23" s="11" t="n"/>
-      <c r="L23" s="11" t="n"/>
-      <c r="M23" s="11" t="n"/>
-      <c r="N23" s="11" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="11" t="n"/>
-      <c r="Q23" s="11" t="n"/>
-      <c r="R23" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>Use unordered_set of ListNode* pointer memory addresses to detect repetition</t>
+        </is>
+      </c>
+      <c r="L23" s="11" t="inlineStr">
+        <is>
+          <t>Had initial doubt on why Floyd fast &amp; slow pointer reset phase works to find exact cycle entry node</t>
+        </is>
+      </c>
+      <c r="M23" s="11" t="inlineStr">
+        <is>
+          <t>Floyd Fast &amp; Slow Pointers (Tortoise &amp; Hare): move slow by 1 step, fast by 2 steps. If fast == slow, cycle exists. Reset slow to head and move both 1 step to find exact cycle entry node.</t>
+        </is>
+      </c>
+      <c r="N23" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>O(1)</t>
+        </is>
+      </c>
+      <c r="P23" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>i know how to make it work but still dont have the exact understanding of it</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 23: Maximum Depth of Binary Tree (Post-order DFS) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -2315,22 +2315,58 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="n"/>
-      <c r="K24" s="11" t="n"/>
-      <c r="L24" s="11" t="n"/>
-      <c r="M24" s="11" t="n"/>
-      <c r="N24" s="11" t="n"/>
-      <c r="O24" s="11" t="n"/>
-      <c r="P24" s="11" t="n"/>
-      <c r="Q24" s="11" t="n"/>
-      <c r="R24" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>Base case current==nullptr return 0, recursive return 1+max(left,right)</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>Rusty on how recursion bubbles up and how to get left/right subtree depths via recursive calls</t>
+        </is>
+      </c>
+      <c r="M24" s="11" t="inlineStr">
+        <is>
+          <t>Tree DFS Post-order: base case root==nullptr returns 0; recurse on left and right subtrees; return 1 + max(leftDepth, rightDepth).</t>
+        </is>
+      </c>
+      <c r="N24" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O24" s="11" t="inlineStr">
+        <is>
+          <t>O(H)</t>
+        </is>
+      </c>
+      <c r="P24" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q24" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr">
+        <is>
+          <t>with practice it will be remembered</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">

</xml_diff>

<commit_message>
Solve No. 24: Validate Binary Search Tree (Range DFS pattern) and sync roadmap tracker
</commit_message>
<xml_diff>
--- a/DSA_Complete_Roadmap_1_to_Interview.xlsx
+++ b/DSA_Complete_Roadmap_1_to_Interview.xlsx
@@ -2399,22 +2399,58 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Solved</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11" t="n"/>
-      <c r="L25" s="11" t="n"/>
-      <c r="M25" s="11" t="n"/>
-      <c r="N25" s="11" t="n"/>
-      <c r="O25" s="11" t="n"/>
-      <c r="P25" s="11" t="n"/>
-      <c r="Q25" s="11" t="n"/>
-      <c r="R25" s="11" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>With Hints</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>Compare node with immediate left and right children</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>Comparing only immediate children misses ancestor violations; had inverted recursive bounds</t>
+        </is>
+      </c>
+      <c r="M25" s="11" t="inlineStr">
+        <is>
+          <t>Recursive DFS with Range Boundaries: validate(node, min_val, max_val) using LLONG_MIN/LLONG_MAX; update upper bound on left child and lower bound on right child</t>
+        </is>
+      </c>
+      <c r="N25" s="11" t="inlineStr">
+        <is>
+          <t>O(N)</t>
+        </is>
+      </c>
+      <c r="O25" s="11" t="inlineStr">
+        <is>
+          <t>O(H)</t>
+        </is>
+      </c>
+      <c r="P25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="inlineStr">
+        <is>
+          <t>revisit again: need to strengthen mental model of recursive range boundaries (min_val, max_val)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">

</xml_diff>